<commit_message>
docs: Update landing page features to reflect recently added Gamification, Notebooks and Avatar features
</commit_message>
<xml_diff>
--- a/Project Tracking.xlsx
+++ b/Project Tracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Leo Harrison\Lucy Tutor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A62B4626-923D-4826-A94E-7A8FA7E3FFE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACE45BAA-2C95-4AB0-9433-D7771A3A54BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="44">
   <si>
     <t>PROJECT PLAN &amp; PROGRESS: ENGLISH AI SYSTEM</t>
   </si>
@@ -150,6 +150,9 @@
   </si>
   <si>
     <t>AI Intergaration</t>
+  </si>
+  <si>
+    <t>Groq AI analyses and explains the result for students in real-time test</t>
   </si>
 </sst>
 </file>
@@ -833,7 +836,7 @@
     <row r="11" spans="2:7" ht="24.6" x14ac:dyDescent="0.25">
       <c r="B11" s="6">
         <f>COUNTA('Detailed Plan'!B5:B35)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C11" s="6">
         <f>COUNTIF('Detailed Plan'!G5:G35, "Completed")</f>
@@ -841,7 +844,7 @@
       </c>
       <c r="D11" s="6">
         <f>COUNTIF('Detailed Plan'!G5:G35, "In Progress")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E11" s="6">
         <f>COUNTIF('Detailed Plan'!G5:G35, "Not Started")</f>
@@ -853,7 +856,7 @@
       </c>
       <c r="G11" s="7">
         <f>AVERAGE('Detailed Plan'!H5:H35)</f>
-        <v>0.12857142857142859</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="14" spans="2:7" ht="19.2" x14ac:dyDescent="0.45">
@@ -907,7 +910,7 @@
       </c>
       <c r="D17" s="11">
         <f>COUNTIF('Detailed Plan'!A5:A35,"PHASE 2")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E17" s="11">
         <f>COUNTIFS('Detailed Plan'!A5:A35,"PHASE 2",'Detailed Plan'!G5:G35,"Completed")</f>
@@ -1228,14 +1231,28 @@
       </c>
     </row>
     <row r="12" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="28"/>
-      <c r="B12" s="34"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="24"/>
+      <c r="A12" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="E12" s="23" t="s">
+        <v>27</v>
+      </c>
       <c r="F12" s="24"/>
-      <c r="G12" s="35"/>
-      <c r="H12" s="26"/>
+      <c r="G12" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="H12" s="31">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="28"/>

</xml_diff>